<commit_message>
Add v0.8.1: subscription plans, profit calculator, Etsy form fix
- Subscription plans modal (Starter/Pro/Power monthly) alongside credit packs
- Profit calculator added to Research tab with reverse Price Finder
- Etsy 2026-04-27 inline-form migration: rewrite selectCategory for new typeahead, require explicit category
- Cross-promo cards for MarkItUp and Marketeer in Account tab
- One-time MarkItUp promo banner on first successful upload
- SEO-tuned manifest name/description, version 0.7.1 → 0.8.1

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/BulkListingPro-template.xlsx
+++ b/templates/BulkListingPro-template.xlsx
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="197">
   <si>
     <t>sku</t>
   </si>
@@ -389,7 +389,7 @@
 - Printable on US Letter &amp; A4</t>
   </si>
   <si>
-    <t>Planners &amp; Templates</t>
+    <t>Planner Templates</t>
   </si>
   <si>
     <t>I did</t>
@@ -473,10 +473,10 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Digital Prints</t>
-  </si>
-  <si>
-    <t>Wall art, printable artwork</t>
+    <t>Digital</t>
+  </si>
+  <si>
+    <t>Digital art, illustrations, wall art (Art &amp; Collectibles &gt; Drawing &amp; Illustration &gt; Digital)</t>
   </si>
   <si>
     <t>Guides &amp; How Tos</t>
@@ -485,19 +485,13 @@
     <t>eBooks, tutorials, instructional guides</t>
   </si>
   <si>
-    <t>Drawing &amp; Illustration</t>
-  </si>
-  <si>
-    <t>Digital art, illustrations, drawings</t>
-  </si>
-  <si>
     <t>Digital Patterns</t>
   </si>
   <si>
     <t>Sewing, knitting, crochet patterns</t>
   </si>
   <si>
-    <t>Daily, weekly, monthly planners and templates</t>
+    <t>Daily, weekly, monthly planner templates</t>
   </si>
   <si>
     <t>Clip Art &amp; Image Files</t>
@@ -506,7 +500,7 @@
     <t>Clipart, PNG bundles, graphic elements</t>
   </si>
   <si>
-    <t>Cutting Machine Files (SVG)</t>
+    <t>Cutting Machine Files</t>
   </si>
   <si>
     <t>SVG files for Cricut, Silhouette</t>
@@ -731,7 +725,7 @@
     <t>5.99</t>
   </si>
   <si>
-    <t>Select from dropdown (see Categories sheet)</t>
+    <t>Must match an Etsy taxonomy LEAF exactly. If unsure, type your term into Etsy's "Find a category" search and copy the bottom of the breadcrumb shown.</t>
   </si>
   <si>
     <t>Who made this product? (select from dropdown)</t>
@@ -795,6 +789,15 @@
   </si>
   <si>
     <t>Save as draft or publish? (select from dropdown)</t>
+  </si>
+  <si>
+    <t>--- CATEGORIES ---</t>
+  </si>
+  <si>
+    <t>Etsy taxonomy:</t>
+  </si>
+  <si>
+    <t>Etsy requires the most-specific (leaf) category name. The Categories sheet lists common digital-product leaves, but Etsy can rename or remove them at any time. If a listing fails on category, type the name into Etsy's "Find a category" search and copy the leaf shown at the end of the breadcrumb.</t>
   </si>
   <si>
     <t>--- FILE PATHS ---</t>
@@ -3044,10 +3047,10 @@
       <formula1>0.2</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Category" error="Please select a category from the dropdown list." sqref="E10:E501">
-      <formula1>Categories!$A$2:$A$25</formula1>
+      <formula1>Categories!$A$2:$A$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Category" error="Please select a category from the dropdown list." sqref="E2:E501">
-      <formula1>Categories!$A$2:$A$25</formula1>
+      <formula1>Categories!$A$2:$A$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Selection" error="Please select from the dropdown." sqref="F10:F501">
       <formula1>"I did,A member of my shop,Another company or person"</formula1>
@@ -3088,7 +3091,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -3129,15 +3132,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
         <v>70</v>
-      </c>
-      <c r="B5" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
         <v>72</v>
@@ -3285,14 +3288,6 @@
       </c>
       <c r="B24" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>109</v>
-      </c>
-      <c r="B25" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -3315,16 +3310,16 @@
   <sheetData>
     <row r="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>112</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>114</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>63</v>
@@ -3332,7 +3327,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -3344,7 +3339,7 @@
         <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -3355,7 +3350,7 @@
         <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D3" t="s">
         <v>59</v>
@@ -3372,7 +3367,7 @@
         <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D4" t="s">
         <v>59</v>
@@ -3383,7 +3378,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -3395,7 +3390,7 @@
         <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -3406,7 +3401,7 @@
         <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D7" t="s">
         <v>59</v>
@@ -3417,7 +3412,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -3429,7 +3424,7 @@
         <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -3440,7 +3435,7 @@
         <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D10" t="s">
         <v>59</v>
@@ -3451,7 +3446,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -3463,7 +3458,7 @@
         <v>40</v>
       </c>
       <c r="E12" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -3474,7 +3469,7 @@
         <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D13" t="s">
         <v>59</v>
@@ -3491,7 +3486,7 @@
         <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D14" t="s">
         <v>59</v>
@@ -3508,7 +3503,7 @@
         <v>59</v>
       </c>
       <c r="C15" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D15" t="s">
         <v>59</v>
@@ -3525,7 +3520,7 @@
         <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D16" t="s">
         <v>59</v>
@@ -3536,7 +3531,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B18" t="s">
         <v>31</v>
@@ -3548,7 +3543,7 @@
         <v>60</v>
       </c>
       <c r="E18" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -3559,7 +3554,7 @@
         <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D19" t="s">
         <v>59</v>
@@ -3570,7 +3565,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B21" t="s">
         <v>32</v>
@@ -3582,7 +3577,7 @@
         <v>61</v>
       </c>
       <c r="E21" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -3593,7 +3588,7 @@
         <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D22" t="s">
         <v>59</v>
@@ -3610,7 +3605,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3622,19 +3617,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>63</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3642,13 +3637,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" t="s">
         <v>140</v>
-      </c>
-      <c r="C2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D2" t="s">
-        <v>142</v>
       </c>
       <c r="E2" t="s">
         <v>59</v>
@@ -3659,13 +3654,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" t="s">
         <v>143</v>
-      </c>
-      <c r="C3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D3" t="s">
-        <v>145</v>
       </c>
       <c r="E3" t="s">
         <v>59</v>
@@ -3676,13 +3671,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E4" t="s">
         <v>59</v>
@@ -3693,13 +3688,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E5" t="s">
         <v>59</v>
@@ -3710,16 +3705,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D6" t="s">
         <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -3727,10 +3722,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D7" t="s">
         <v>37</v>
@@ -3744,10 +3739,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D8" t="s">
         <v>38</v>
@@ -3761,10 +3756,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D9" t="s">
         <v>39</v>
@@ -3778,10 +3773,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D10" t="s">
         <v>40</v>
@@ -3795,13 +3790,13 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E11" t="s">
         <v>59</v>
@@ -3809,13 +3804,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D12" t="s">
         <v>59</v>
@@ -3829,13 +3824,13 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C13" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D13" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E13" t="s">
         <v>59</v>
@@ -3846,13 +3841,13 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E14" t="s">
         <v>59</v>
@@ -3860,16 +3855,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>161</v>
+      </c>
+      <c r="B15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" t="s">
+        <v>162</v>
+      </c>
+      <c r="D15" t="s">
         <v>163</v>
-      </c>
-      <c r="B15" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15" t="s">
-        <v>164</v>
-      </c>
-      <c r="D15" t="s">
-        <v>165</v>
       </c>
       <c r="E15" t="s">
         <v>59</v>
@@ -3880,13 +3875,13 @@
         <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C16" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E16" t="s">
         <v>59</v>
@@ -3897,16 +3892,16 @@
         <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C17" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D17" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E17" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -3914,10 +3909,10 @@
         <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D18" t="s">
         <v>60</v>
@@ -3931,10 +3926,10 @@
         <v>32</v>
       </c>
       <c r="B19" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C19" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D19" t="s">
         <v>61</v>
@@ -3945,31 +3940,44 @@
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>171</v>
+      </c>
+      <c r="C22" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>173</v>
       </c>
-      <c r="C22" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="C25" t="s">
         <v>175</v>
       </c>
-      <c r="C23" t="s">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="C26" t="s">
         <v>177</v>
       </c>
-      <c r="C24" t="s">
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>178</v>
+      </c>
+      <c r="C27" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -3989,18 +3997,18 @@
   <sheetData>
     <row r="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -4008,7 +4016,7 @@
         <v>59</v>
       </c>
       <c r="B3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -4016,7 +4024,7 @@
         <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -4024,15 +4032,15 @@
         <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -4040,7 +4048,7 @@
         <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -4048,7 +4056,7 @@
         <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -4056,15 +4064,15 @@
         <v>59</v>
       </c>
       <c r="B10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B12" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -4072,7 +4080,7 @@
         <v>59</v>
       </c>
       <c r="B13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -4080,7 +4088,7 @@
         <v>59</v>
       </c>
       <c r="B14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -4088,7 +4096,7 @@
         <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>